<commit_message>
fix(school-forms): correct SF1, SF5, and SF9 draft exports
- Fill SF1 birth province only from confirmed Philippine data.
- Leave SF5 general averages for adviser entry and add DepEd LIS proficiency-band warnings to previews and downloads.
- Replace the app’s SF9 copy with the supplied three-term layout, remap its grade cells, and leave unsupported grades blank for adviser review.
- Update SF9 mapping metadata and overflow editing; remove the false preview-limit warning.
- Expand school-form regression coverage.
</commit_message>
<xml_diff>
--- a/assets/templates/school-forms/sf9.xlsx
+++ b/assets/templates/school-forms/sf9.xlsx
@@ -2798,13 +2798,14 @@
       </c>
       <c r="G30" s="110"/>
       <c r="H30" s="110"/>
-      <c r="J30" s="137" t="s">
+      <c r="I30" s="137" t="s">
         <v>23</v>
       </c>
-      <c r="K30" s="110" t="s">
+      <c r="J30" s="110" t="s">
         <v>63</v>
       </c>
-      <c r="L30" s="110"/>
+      <c r="K30" s="110"/>
+      <c r="L30" s="47"/>
       <c r="M30" s="48"/>
       <c r="N30" s="48"/>
       <c r="O30" s="49"/>
@@ -2843,14 +2844,10 @@
       <c r="H31" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="I31" s="67" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="J31" s="137"/>
+      <c r="I31" s="137"/>
+      <c r="J31" s="110"/>
       <c r="K31" s="110"/>
-      <c r="L31" s="110"/>
+      <c r="L31" s="11"/>
       <c r="M31" s="12"/>
       <c r="N31" s="12"/>
       <c r="O31" s="10"/>
@@ -2883,10 +2880,10 @@
       <c r="F32" s="68"/>
       <c r="G32" s="68"/>
       <c r="H32" s="68"/>
-      <c r="I32" s="68"/>
-      <c r="J32" s="65"/>
+      <c r="I32" s="65"/>
+      <c r="J32" s="101"/>
       <c r="K32" s="101"/>
-      <c r="L32" s="101"/>
+      <c r="L32" s="11"/>
       <c r="M32" s="12"/>
       <c r="N32" s="12"/>
       <c r="O32" s="10"/>
@@ -2906,10 +2903,10 @@
       <c r="F33" s="68"/>
       <c r="G33" s="68"/>
       <c r="H33" s="68"/>
-      <c r="I33" s="68"/>
-      <c r="J33" s="65"/>
+      <c r="I33" s="65"/>
+      <c r="J33" s="101"/>
       <c r="K33" s="101"/>
-      <c r="L33" s="101"/>
+      <c r="L33" s="11"/>
       <c r="M33" s="12"/>
       <c r="N33" s="12"/>
       <c r="O33" s="10"/>
@@ -2942,10 +2939,10 @@
       <c r="F34" s="68"/>
       <c r="G34" s="68"/>
       <c r="H34" s="68"/>
-      <c r="I34" s="68"/>
-      <c r="J34" s="65"/>
+      <c r="I34" s="65"/>
+      <c r="J34" s="101"/>
       <c r="K34" s="101"/>
-      <c r="L34" s="101"/>
+      <c r="L34" s="11"/>
       <c r="M34" s="12"/>
       <c r="N34" s="12"/>
       <c r="O34" s="10"/>
@@ -2978,10 +2975,10 @@
       <c r="F35" s="68"/>
       <c r="G35" s="68"/>
       <c r="H35" s="68"/>
-      <c r="I35" s="68"/>
-      <c r="J35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="101"/>
       <c r="K35" s="101"/>
-      <c r="L35" s="101"/>
+      <c r="L35" s="11"/>
       <c r="M35" s="12"/>
       <c r="N35" s="12"/>
       <c r="O35" s="10"/>
@@ -3014,10 +3011,10 @@
       <c r="F36" s="68"/>
       <c r="G36" s="68"/>
       <c r="H36" s="68"/>
-      <c r="I36" s="68"/>
-      <c r="J36" s="65"/>
+      <c r="I36" s="65"/>
+      <c r="J36" s="101"/>
       <c r="K36" s="101"/>
-      <c r="L36" s="101"/>
+      <c r="L36" s="11"/>
       <c r="M36" s="12"/>
       <c r="N36" s="12"/>
       <c r="O36" s="10"/>
@@ -3048,10 +3045,10 @@
       <c r="F37" s="68"/>
       <c r="G37" s="68"/>
       <c r="H37" s="68"/>
-      <c r="I37" s="68"/>
-      <c r="J37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="101"/>
       <c r="K37" s="101"/>
-      <c r="L37" s="101"/>
+      <c r="L37" s="11"/>
       <c r="M37" s="12"/>
       <c r="N37" s="12"/>
       <c r="O37" s="10"/>
@@ -3084,10 +3081,10 @@
       <c r="F38" s="69"/>
       <c r="G38" s="69"/>
       <c r="H38" s="69"/>
-      <c r="I38" s="69"/>
-      <c r="J38" s="65"/>
+      <c r="I38" s="65"/>
+      <c r="J38" s="101"/>
       <c r="K38" s="101"/>
-      <c r="L38" s="101"/>
+      <c r="L38" s="11"/>
       <c r="M38" s="12"/>
       <c r="N38" s="12"/>
       <c r="O38" s="10"/>
@@ -3120,10 +3117,10 @@
       <c r="F39" s="68"/>
       <c r="G39" s="68"/>
       <c r="H39" s="68"/>
-      <c r="I39" s="68"/>
-      <c r="J39" s="65"/>
+      <c r="I39" s="65"/>
+      <c r="J39" s="101"/>
       <c r="K39" s="101"/>
-      <c r="L39" s="101"/>
+      <c r="L39" s="14"/>
       <c r="M39" s="8"/>
       <c r="N39" s="8"/>
       <c r="O39" s="4"/>
@@ -3154,10 +3151,10 @@
       <c r="F40" s="68"/>
       <c r="G40" s="70"/>
       <c r="H40" s="70"/>
-      <c r="I40" s="70"/>
-      <c r="J40" s="65"/>
+      <c r="I40" s="65"/>
+      <c r="J40" s="109"/>
       <c r="K40" s="109"/>
-      <c r="L40" s="109"/>
+      <c r="L40" s="14"/>
       <c r="M40" s="8"/>
       <c r="N40" s="8"/>
       <c r="O40" s="4"/>
@@ -3190,10 +3187,10 @@
       <c r="F41" s="69"/>
       <c r="G41" s="69"/>
       <c r="H41" s="69"/>
-      <c r="I41" s="69"/>
-      <c r="J41" s="65"/>
+      <c r="I41" s="65"/>
+      <c r="J41" s="110"/>
       <c r="K41" s="110"/>
-      <c r="L41" s="110"/>
+      <c r="L41" s="14"/>
       <c r="M41" s="8"/>
       <c r="N41" s="8"/>
       <c r="O41" s="4"/>
@@ -3228,9 +3225,10 @@
       <c r="F42" s="92"/>
       <c r="G42" s="92"/>
       <c r="H42" s="92"/>
-      <c r="J42" s="93"/>
+      <c r="I42" s="93"/>
+      <c r="J42" s="94"/>
       <c r="K42" s="94"/>
-      <c r="L42" s="94"/>
+      <c r="L42" s="14"/>
       <c r="M42" s="8"/>
       <c r="N42" s="8"/>
       <c r="O42" s="4"/>
@@ -3260,9 +3258,10 @@
       <c r="F43" s="92"/>
       <c r="G43" s="92"/>
       <c r="H43" s="92"/>
-      <c r="J43" s="93"/>
+      <c r="I43" s="93"/>
+      <c r="J43" s="94"/>
       <c r="K43" s="94"/>
-      <c r="L43" s="94"/>
+      <c r="L43" s="14"/>
       <c r="M43" s="8"/>
       <c r="N43" s="8"/>
       <c r="O43" s="4"/>
@@ -34223,10 +34222,10 @@
   <mergeCells count="125">
     <mergeCell ref="Q44:AC44"/>
     <mergeCell ref="H27:K27"/>
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="J30:J31"/>
-    <mergeCell ref="K30:L31"/>
-    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="J30:K31"/>
+    <mergeCell ref="J32:K32"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="H28:K28"/>
@@ -34235,10 +34234,10 @@
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B34:E34"/>
     <mergeCell ref="B35:E35"/>
-    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="J39:K39"/>
     <mergeCell ref="B38:E38"/>
     <mergeCell ref="B39:E39"/>
-    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="J38:K38"/>
     <mergeCell ref="B29:K29"/>
     <mergeCell ref="B30:E31"/>
     <mergeCell ref="B32:E32"/>
@@ -34308,11 +34307,11 @@
     <mergeCell ref="Q45:AC45"/>
     <mergeCell ref="B9:K9"/>
     <mergeCell ref="C18:E18"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="J37:K37"/>
     <mergeCell ref="B14:K14"/>
     <mergeCell ref="C17:G17"/>
     <mergeCell ref="B21:C21"/>
@@ -34321,8 +34320,8 @@
     <mergeCell ref="B10:K10"/>
     <mergeCell ref="F45:G45"/>
     <mergeCell ref="I45:J45"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J41:K41"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="I47:J47"/>
     <mergeCell ref="I48:J48"/>
@@ -34332,8 +34331,8 @@
     <mergeCell ref="I51:J51"/>
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B42:H43"/>
-    <mergeCell ref="J42:J43"/>
-    <mergeCell ref="K42:L43"/>
+    <mergeCell ref="I42:I43"/>
+    <mergeCell ref="J42:K43"/>
     <mergeCell ref="I50:J50"/>
     <mergeCell ref="C49:E49"/>
     <mergeCell ref="F49:G49"/>

</xml_diff>